<commit_message>
Sync local training data and review docs
</commit_message>
<xml_diff>
--- a/Training Data/Automation/LCL.xlsx
+++ b/Training Data/Automation/LCL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\SMS_Automation\Training Data\Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78C767D-7DE7-4CE9-8D2B-9937C6CBFBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7AE9EE-B388-41F2-BE06-045CE489DDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LCL" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="139">
-  <si>
-    <t>SL No</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
   <si>
     <t>Request</t>
   </si>
@@ -31,412 +28,315 @@
     <t>Reply</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>LCL 01617610134</t>
   </si>
   <si>
-    <t>MSISDN: 8801617610134, MSISDN B Party: 8801723599495, Last Call location: Ward No 24, BARISAL SADAR KOTWALI, Barisal, LAC ID: 8005, Cell ID: 28196, Lat_Long: 22.66143, 90.3495, Date_time: 20260607205630, IMEI: 860068048764800, IMSI: 470075012337288 [Robi] | RADIO LOCATION: Ward No-24, Barisal Sadar (kotwali), Barisal, LAC ID: 8005, CELL ID: 28196, LAT, LONG: 22.66143, 90.3495, MS STATUS: Attached, LAST ACTION TIME: 2026-06-07 21:37:12 [Robi]</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>LCL 01724034442</t>
   </si>
   <si>
-    <t>8801724034442, GP 2560MB, SMSMT, 06/06/2026 10:09:30, [48231 29700639], NALCHITY, JHALOKATHI, IMEI: 352931900461140, IMSI: 470010499560912 [GP] | No RL Info Found of 1724034442 [GP]</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>LCL 01316178945</t>
   </si>
   <si>
-    <t>8801316178945 / 8801323428959, MTC, 07/06/2026 19:49:15, [23093 53640], PASCHIM CHAR DAPDAPIA, DAPDAPIA, NALCHITY, JHALOKATI, IMEI: 868236085902400, IMSI: 470010491153713 [GP] | MSISDN: 8801316178945, LastActiveDateTime: 2026-06-07 22:30:50, LACID: 48261, CellID: 35855137, Latitude: 22.658194, Longitude: 90.344889, Address: 13, PARARA ROAD, P.S. KOTOWALI, DIST. BARISAL, CS Status: Idle [GP]</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>LCL 01779398037</t>
   </si>
   <si>
-    <t>8801779398037, 4750, SMSMT, 07/06/2026 23:25:34, [56312 25735199], HOLDING NO. 54/1, FAKIRAPUL, DHAKA, IMEI: 359127131839920, IMSI: 470010441603444 [GP] | MSISDN: 8801779398037, LastActiveDateTime: 2026-06-07 23:35:36, LACID: 56312, CellID: 25850635, Latitude: 23.735361, Longitude: 90.416222, Address: 38, NAYAPALTAN, DHAKA-1000, CS Status: Idle [GP]</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>LCL 01312123075</t>
   </si>
   <si>
     <t>8801312123075 / 8801620479563, MTC, 07/06/2026 14:01:06, [27007 22290], VILL ANGARIA, P.O ANGARIA BONDOR, UNION 4 ANGARIA, P.S. DUMKI, PATUAKHALI, IMEI: 357146190845460, IMSI: 470010318024314 [GP]</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>LCL 01620479563</t>
   </si>
   <si>
     <t>MSISDN: 8801620479563, MSISDN B Party: 8801621603027, Last Call location: Vill Bhorpasha, PS Bakerganj, Barishal, LAC ID: 8005, Cell ID: 3610, Lat_Long: 22.5189, 90.343, Date_time: 20260608011153, IMEI: 354680100182050, IMSI: 470075028693785 [Robi]</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
     <t>LCL 01775494991</t>
   </si>
   <si>
     <t>8801775494991 / 8801755370218, MTC, 03/06/2026 15:18:11, [46361 28989246], VILL P.O DHAMURA, UNION SHOLOK, P.S UZIRPUR, DIST BARISAL, IMEI: 868126062531170, IMSI: 470010444160092 [GP]</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>LCL 01333061009</t>
   </si>
   <si>
     <t>8801333061009, GP 35MIN, SMSMT, 03/06/2026 11:08:05, [46361 28989200], VILL P.O DHAMURA, UNION SHOLOK, P.S UZIRPUR, DIST BARISAL, IMEI: 868126062531160, IMSI: 470010426256901 [GP]</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
     <t>LCL 01755370218</t>
   </si>
   <si>
     <t>(B-party of 01775494991 - included in batch reply above)</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>LCL 01958395882</t>
   </si>
   <si>
     <t>MSISDN: 8801958395882, Datetime: 20260608104540, LAC ID: 673, Cell ID: 47113, Address: Vill: Omorpur, Post: Bhuiyarhat, PS: Charfashio, Dist: Bhola, BPARTY: 8801901900977, IMEI: 354388221566410, IMSI: 470039215027744, UsageType: SMSMT, NetworkType: 2G. - Banglalink</t>
   </si>
   <si>
-    <t>11</t>
-  </si>
-  <si>
     <t>LCL 01931270994</t>
   </si>
   <si>
     <t>MSISDN: 8801931270994, Datetime: 20260607122312, LAC ID: 6030, Cell ID: 15425873, Address: Barothi Bazar, Gaurnadi, Barisal, BPARTY: 880424c204468616, IMEI: 350789590248680, IMSI: 470039926367303, UsageType: SMSMT, NetworkType: 4G. - Banglalink</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
     <t>LCL 01567847825</t>
   </si>
   <si>
     <t>(No reply visible in loaded messages)</t>
   </si>
   <si>
-    <t>13</t>
-  </si>
-  <si>
     <t>LCL 01811426571</t>
   </si>
   <si>
     <t>MSISDN: 8801811426571, MSISDN B Party: 4A686F74706F744C6F61, Last Call location: Ward No 46 Part, Hazaribagh, Dhaka, LAC ID: 407, Cell ID: 46478, Lat_Long: 23.75, 90.3448, Date_time: 20260608140235, IMEI: 351207980537560, IMSI: 470022557928135 [Robi]</t>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
     <t>LCL 01730911057</t>
   </si>
   <si>
     <t>8801730911057, GP 45MIN, SMSMT, 08/06/2026 13:27:23, [21034 42832], NEAR BASILA GARDEN CITY PLAY GROUND, MOHAMMADPUR, IMEI: 351207980537570, IMSI: 470010314611892 [GP]</t>
   </si>
   <si>
-    <t>15</t>
-  </si>
-  <si>
     <t>LCL 01750193604</t>
   </si>
   <si>
     <t>8801750193604 / 8801337510464, MTC, 04/06/2026 16:33:43, [23022 50587], RAMNAGAR, MAHESHPUR, BAKORGANJ, BARISAL, IMEI: 865455059456460, IMSI: 470010513871161 [GP]</t>
   </si>
   <si>
-    <t>16</t>
-  </si>
-  <si>
     <t>LCL 01862303409</t>
   </si>
   <si>
     <t>(Part of Mahendigang batch - reply not separately visible)</t>
   </si>
   <si>
-    <t>17</t>
-  </si>
-  <si>
     <t>LCL 01612268083</t>
   </si>
   <si>
     <t>MSISDN: 8801612268083, MSISDN B Party: 8801903311869, Last Call location: Kashipur, Narayanganj Sadar, Narayanganj, LAC ID: 30024, Cell ID: 7842, Lat_Long: 23.60738, 90.491606, Date_time: 20260607012317, IMEI: 351600344667680, IMSI: 470075031845935 [Robi]</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
     <t>LCL 01719698577</t>
   </si>
   <si>
     <t>8801719698577 / 8801732454040, MOC, 08/06/2026 12:26:22, [48251 35844643], ANEX BHABAN, BARISAL CITY CORPORATION, BIBIRPUKUR, BARISAL SADAR, BARISAL, IMEI: 868477051245710, IMSI: 470010494597953 [GP]</t>
   </si>
   <si>
-    <t>19</t>
-  </si>
-  <si>
     <t>LCL 01919904263</t>
   </si>
   <si>
     <t>MN: 01919904263 No Radio Location Found. - Banglalink | MSISDN: 8801919904263, Datetime: 20260605152339, LAC ID: 680, Cell ID: 46521, Address: Vill: Hayatsar, PO: Churamon, PS: Kawnia, Dist: Barisal, IMEI: 864434060146480, IMSI: 470039934828149, NetworkType: 2G. - Banglalink</t>
   </si>
   <si>
-    <t>20</t>
-  </si>
-  <si>
     <t>LCL 01315607014</t>
   </si>
   <si>
     <t>8801315607014 / 8801717167974, MTC, 09/06/2026 00:13:20, [21037 46256], 182/1, EAST TEJTURI BAZAR, TEJGAON, DHAKA, IMSI: 470010459858472 [GP]</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
     <t>LCL 01760675453</t>
   </si>
   <si>
     <t>Sorry No records found against this number 1760675453 [GP]</t>
   </si>
   <si>
-    <t>22</t>
-  </si>
-  <si>
     <t>LCL 01758696171</t>
   </si>
   <si>
     <t>8801758696171, 4750, SMSMT, 22/04/2026 17:47:00, [46501 28984589], KOLCHORI SHAMRAI, CHANPUR, MAHENDIGANJ, BARISAL, IMEI: 353522649744610, IMSI: 470010632925146 [GP]</t>
   </si>
   <si>
-    <t>23</t>
-  </si>
-  <si>
     <t>LCL 01310648009</t>
   </si>
   <si>
     <t>Sorry No records found against this number 1310648009 [GP]</t>
   </si>
   <si>
-    <t>24</t>
-  </si>
-  <si>
     <t>LCL 01721305809</t>
   </si>
   <si>
     <t>Sorry No records found against this number 1721305809 [GP]</t>
   </si>
   <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>LCL 01741989106</t>
-  </si>
-  <si>
-    <t>(LCL 01711989106 - reply not visible)</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>LCL 01863308890</t>
-  </si>
-  <si>
-    <t>(Reply not visible for this request)</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>LCL 01345636569</t>
-  </si>
-  <si>
-    <t>8801345636569 / 8801610656389, MTC, 09/06/2026 13:29:03, [25049 11311], ADAMJEE ROAD (IQBAL GROUP OF INDUSTRIES), P.S: SHIDDHIRGANJ, NARAYANGANJ, IMEI: 861407080007970, IMSI: 470010507001900 [GP]</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>LCL 01715116016</t>
-  </si>
-  <si>
-    <t>8801715116016 / 8801798460306, MTC, 09/06/2026 23:50:36, [23047 13696], 108/102 NATUN BAZAR, BARISHAL, BARISHAL SADAR, BARISAL, IMEI: 860366069821140, IMSI: 470010553967042 [GP] | MSISDN: 8801715116016, LastActiveDateTime: 2026-06-10 00:23:42, LACID: 46331, CellID: 35873311, Latitude: 22.805417, Longitude: 90.309056, Address: FACULTY OF ANIMAL SCIENCE AND VETERINARY MEDICINE BUILDING, RAHOMOTPUR, BABUGANJ, BARISAL, CS Status: Idle [GP]</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
     <t>LCL 01911152692</t>
   </si>
   <si>
     <t>MSISDN: 8801911152692, Datetime: 20260609104730, LAC ID: 680, Cell ID: 60282, Address: Vill - Kandihar, Thana - Banaripara, District - Barisal, BPARTY: 880624B617368, IMEI: 354496311003140, IMSI: 470037400048620, UsageType: SMSMT, NetworkType: 2G. - Banglalink</t>
   </si>
   <si>
-    <t>30</t>
-  </si>
-  <si>
     <t>LCL 01711207942</t>
   </si>
   <si>
     <t>8801711207942, MyGP, SMSMT, 09/06/2026 10:47:36, [46341 29604875], BANORIPARA, BARISAL, IMEI: 354496311038860, IMSI: 470010440738577 [GP]</t>
   </si>
   <si>
-    <t>31</t>
-  </si>
-  <si>
     <t>LCL 01631371920</t>
   </si>
   <si>
     <t>MSISDN: 8801631371920, MSISDN B Party: Airtel, Last Call location: vill Tetla, P O Tetla, Banaripara, Barishal, LAC ID: 820043, Cell ID: 75, Lat_Long: 22.81357, 90.08629, Date_time: 20260605072416, IMEI: 862410074377150, IMSI: 470075005033851 [Robi]</t>
   </si>
   <si>
-    <t>32</t>
-  </si>
-  <si>
     <t>LCL 01711351928</t>
   </si>
   <si>
     <t>8801711351928, Navana Land, SMSMT, 10/06/2026 10:15:20, [62411 40979232], MUNICIPAL HOLDING NO. 59/B/1, ROY J. C. GUHA ROAD, KRISHTOPUR, P.S MYMENSINGH SADAR, MYMENSINGH, IMEI: 862365044189750, IMSI: 470010513636040 [GP]</t>
   </si>
   <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>LCL 01888002490</t>
-  </si>
-  <si>
-    <t>(Split from multi-number request LCL 01888002490 01333821028 - reply not separately shown)</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>LCL 01333821028</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
     <t>LCL 01937344944</t>
   </si>
   <si>
     <t>MSISDN: 8801937344944, Datetime: 20260608111805, LAC ID: 461, Cell ID: 41753, Address: House No: 105/22k, Thana Road, PS: Sonadanga, Dist: Khulna, BPARTY: 8801938773957, IMEI: 359498701015280, IMSI: 470039946221263, UsageType: MTC, NetworkType: 2G. - Banglalink</t>
   </si>
   <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>LCL 01623766981</t>
-  </si>
-  <si>
-    <t>(No reply visible for this request)</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>LCL 01720542190</t>
-  </si>
-  <si>
-    <t>8801720542190 / 8801725927837, MOC, 10/06/2026 09:48:00, [23126 50574], VILL KADIRABAD, P.O KADIRABAD, UNION LATA, P.S MAHENDIGANJ, BARISAL, IMEI: 344685625789860, IMSI: 470010383180005 [GP]</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
     <t>LCL 01703520704</t>
   </si>
   <si>
     <t>8801703520704, GP, SMSMT, 09/06/2026 18:13:41, [46301 28995871], VILL-GABIKHOLA, P.O-GARURIA, P/S-BAKERGONJ, BARISAL, IMEI: 866446059282170, IMSI: 470010491639968 [GP]</t>
   </si>
   <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>LCL 01602-389949</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>LCL 01719182914</t>
-  </si>
-  <si>
-    <t>8801719182914 / 8801789360756, MTC, 09/06/2026 23:10:54, [23126 29095], PATTANI BHANGAR CHAR, GUABARIA, HIZLA, BARISHAL, IMSI: 470010352788437 [GP]</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>43</t>
-  </si>
-  <si>
-    <t>LCL 01757265392</t>
-  </si>
-  <si>
-    <t>(Split from 5-number batch: LCL 01757265392 01844468499 01768233922 01736373112 01757232333 - system returned batch reply for these numbers)</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>LCL 01844468499</t>
-  </si>
-  <si>
-    <t>(Split from 5-number batch - see above)</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>LCL 01768233922</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>LCL 01736373112</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>LCL 01757232333</t>
-  </si>
-  <si>
-    <t>8801724761972 / 8801325397520, MTC, 10/06/2026 21:58:49, [22049 50739], MOUZA-BANARIPARA, SADAR ROAD, 3 NO WORD, BANARIPARA, BARISHAL, IMEI: 350419993156990, IMSI: 470010081907258 [GP]</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
     <t>LCL 01319472535</t>
   </si>
   <si>
-    <t>MSISDN: 8801319472535, LastActiveDateTime: 2026-06-10 12:31:29, LACID: 23066, CellID: 22578, Latitude: 23.371472, Longitude: 90.034444, Address: VILL.- RASHIBPURA, MALIGRAM BAZAR, MOUZA-MALIGRAM, VANGA, FARIDPUR, CS Status: Idle, Volte Status: N/A [GP] | 8801319472535, GP, SMSMT, 10/06/2026 12:31:17, [48271 28698401], VILL: PULIA, P.O: CHANDRA BAZAR, UNION: CHANDRA, P.S: BHANGA, FARIDPUR, IMEI: 357726270741110, IMSI: 470010402936218 [GP]</t>
+    <t>MSISDN: 8801617610134, MSISDN B Party: 8801723599495, Last Call location: Ward No 24, BARISAL SADAR KOTWALI, Barisal, LAC ID: 8005, Cell ID: 28196, Lat_Long: 22.66143, 90.3495, Date_time: 20260607205630, IMEI: 860068048764800, IMSI: 470075012337288 [Robi] |</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8801724034442, GP 2560MB, SMSMT, 06/06/2026 10:09:30, [48231 29700639], NALCHITY, JHALOKATHI, IMEI: 352931900461140, IMSI: 470010499560912 [GP] | </t>
+  </si>
+  <si>
+    <t>MSISDN: 8801316178945, LastActiveDateTime: 2026-06-07 22:30:50, LACID: 48261, CellID: 35855137, Latitude: 22.658194, Longitude: 90.344889, Address: 13, PARARA ROAD, P.S. KOTOWALI, DIST. BARISAL, CS Status: Idle [GP]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8801779398037, 4750, SMSMT, 07/06/2026 23:25:34, [56312 25735199], HOLDING NO. 54/1, FAKIRAPUL, DHAKA, IMEI: 359127131839920, IMSI: 470010441603444 [GP] | </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSISDN: 8801319472535, LastActiveDateTime: 2026-06-10 12:31:29, LACID: 23066, CellID: 22578, Latitude: 23.371472, Longitude: 90.034444, Address: VILL.- RASHIBPURA, MALIGRAM BAZAR, MOUZA-MALIGRAM, VANGA, FARIDPUR, CS Status: Idle, Volte Status: N/A [GP] | </t>
+  </si>
+  <si>
+    <t>LCL 01864591168</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801864591168
+MSISDN B Party: 8801821764035
+Last Call location: Castle Green,H  142,Green Road,,Farmgate,Dhaka 1215
+LAC ID: 108
+Cell ID: 897
+Lat_Long: 23.7535, 90.3882
+Date_time: 20260615204215
+IMEI: 869727086437610
+IMSI: 470022563349762 [Robi]</t>
+  </si>
+  <si>
+    <t>LCL 01305424184</t>
+  </si>
+  <si>
+    <t>8801305424184
+8801933640177
+MOC
+15/06/2026 09:26:42
+[23117 22339]
+MOUZA NAGARBAKA,  P.S. &amp;amp; SUB REGISTRY OFFICE MIRPUR,  DIST. KUSTIA.
+866941062115380
+470010485077007 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01721586862</t>
+  </si>
+  <si>
+    <t>8801721586862
+8801932161211
+MTC
+15/06/2026 20:32:11
+[23011 21691]
+BISWAS BARI, VILL-LOKKHIKOL,  P.S. JHENAIDAH SADAR,  JHENAIDAH JHENAIDAH SADAR  JHENAIDAH
+358564994871350
+470010483500257 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01744708168</t>
+  </si>
+  <si>
+    <t>8801744708168
+bKash
+SMSMT
+14/06/2026 19:57:22
+[21025 12297]
+VILL: SHEMPUR  HEMAYETPUR PS: SAVER  DIST: DHAKA
+353973860706950
+470010369479393 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01836526001</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801836526001
+MSISDN B Party: 5370656369616C506163
+Last Call location: Vill  Purbakandi Paschimpar, P O  Uttar Char   8270, P S  Mehendiganj, Dist  Barisal
+LAC ID: 8006
+Cell ID: 28390
+Lat_Long: 22.85657, 90.54667
+Date_time: 20251202132329
+IMEI: 866254085016420
+IMSI: 470022595759345 [Robi]</t>
+  </si>
+  <si>
+    <t>LCL 01994076892</t>
+  </si>
+  <si>
+    <t>MSISDN: 01994076892 No Data Available within 90 Days (LCL) - Banglalink</t>
+  </si>
+  <si>
+    <t>LCL 01759778356</t>
+  </si>
+  <si>
+    <t>Sorry No records found against this number 1759778356 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01938218511</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801938218511, Datetime: 20260615224027, LAC ID: 1202, Cell ID: 3012355, Address: Md. Abul Kashem, 311 south Monipur (Mollapara), Near Kuwaity mosque, Mirpur-2, BPARTY: 880811660038123, IMEI: 350347640688710, IMSI: 470039954420135, UsageType: MTC, NetworkType: 4G. - Banglalink</t>
+  </si>
+  <si>
+    <t>LCL 01309821052</t>
+  </si>
+  <si>
+    <t>8801309821052
+8801729558492
+MOC
+15/06/2026 17:13:57
+[23047 50689]
+APON NIBASH, HOUSE NO# 502, ROAD- AGARPUR,BARISHAL SADAR,BARISHAL SADAR,BARISHAL
+356008090251500
+470010482120610 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01340484381</t>
+  </si>
+  <si>
+    <t>LCL 01869033806</t>
+  </si>
+  <si>
+    <t>Sorry No records found against this number 1869033806 [GP]</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>**Look this number is robi but msg sent to gp. So no record replied</t>
+  </si>
+  <si>
+    <t>8801340484381
+8801847348716
+SMSMT
+16/06/2026 13:31:07
+[48251 2244188]
+866183068507830
+470010977470798 [GP]</t>
+  </si>
+  <si>
+    <t>SL NO</t>
   </si>
 </sst>
 </file>
@@ -579,7 +479,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -759,8 +659,20 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -875,6 +787,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -920,16 +845,22 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -976,15 +907,12 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1000,12 +928,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}" name="Table1" displayName="Table1" ref="A1:C49" totalsRowShown="0">
-  <autoFilter ref="A1:C49" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}" name="Table1" displayName="Table1" ref="B1:D46" totalsRowShown="0">
+  <autoFilter ref="B1:D46" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{325C3C9D-4760-4419-9DD2-AB65634C7B08}" name="SL No" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{2D7AC2AD-014A-48FF-95F7-9CC4728A926F}" name="Request" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{3864D13E-23B2-4E39-A10E-6D64B9F5D0CF}" name="Reply" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{3C8B4891-26D5-4D39-A506-E466FD96FCE7}" name="Column1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1328,551 +1256,524 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="A1:D46"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="8.83984375" style="1"/>
-    <col min="2" max="2" width="19.1015625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="62.7890625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="19.08984375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="69.54296875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="51.58984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A1" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="100.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="1" t="s">
+      <c r="C2" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C3" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C4" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="1" t="s">
+      <c r="C5" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="86.4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="86.4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="1" t="s">
+    <row r="9" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="1" t="s">
+    <row r="12" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="3" t="s">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A13" s="5">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="1" t="s">
+      <c r="C13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="2" t="s">
+    </row>
+    <row r="14" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="1" t="s">
+    <row r="15" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A15" s="5">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="3" t="s">
+    </row>
+    <row r="16" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="1" t="s">
+      <c r="C16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="2" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A17" s="5">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="1" t="s">
+    <row r="18" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="3" t="s">
+    </row>
+    <row r="19" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A19" s="5">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="1" t="s">
+      <c r="C19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="2" t="s">
+    </row>
+    <row r="20" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="1" t="s">
+    <row r="21" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A21" s="5">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="3" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A22" s="4">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="1" t="s">
+      <c r="C22" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="2" t="s">
+    </row>
+    <row r="23" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A23" s="5">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C23" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="1" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A24" s="4">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="3" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A25" s="5">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="1" t="s">
+      <c r="C25" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="2" t="s">
+    </row>
+    <row r="26" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C26" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="1" t="s">
+    <row r="27" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A27" s="5">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="3" t="s">
+    </row>
+    <row r="28" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="2" t="s">
+    </row>
+    <row r="29" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A29" s="5">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C29" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="1" t="s">
+    <row r="30" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A30" s="4">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="3" t="s">
+    </row>
+    <row r="31" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A31" s="5">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="1" t="s">
+      <c r="C31" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="2" t="s">
+    </row>
+    <row r="32" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A32" s="4">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="1" t="s">
+      <c r="C32" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="2" t="s">
+    </row>
+    <row r="33" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A33" s="5">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C33" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="1" t="s">
+    <row r="34" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+      <c r="A34" s="4">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="3" t="s">
+    </row>
+    <row r="35" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A35" s="5">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="1" t="s">
+      <c r="C35" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B24" s="2" t="s">
+    </row>
+    <row r="36" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+      <c r="A36" s="4">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C36" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="1" t="s">
+    <row r="37" spans="1:4" ht="147.5" x14ac:dyDescent="0.75">
+      <c r="A37" s="5">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="3" t="s">
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A38" s="4">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="1" t="s">
+      <c r="C38" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B26" s="2" t="s">
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A39" s="5">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C39" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="1" t="s">
+    <row r="40" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A40" s="4">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C27" s="3" t="s">
+    </row>
+    <row r="41" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+      <c r="A41" s="5">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A42" s="4">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="1" t="s">
+      <c r="C42" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B28" s="2" t="s">
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A43" s="5">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D43" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="103.25" x14ac:dyDescent="0.75">
+      <c r="A44" s="4">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="100.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="1" t="s">
+      <c r="C44" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C34" s="3" t="s">
+    </row>
+    <row r="45" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A45" s="5">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="B43" s="2" t="s">
+      <c r="C45" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="103.25" x14ac:dyDescent="0.75">
+      <c r="A46" s="4">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C43" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" ht="100.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>138</v>
+      <c r="C46" s="2" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use curated workbooks for reply matching
</commit_message>
<xml_diff>
--- a/Training Data/Automation/LCL.xlsx
+++ b/Training Data/Automation/LCL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\SMS_Automation\Training Data\Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7AE9EE-B388-41F2-BE06-045CE489DDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECBD642C-916B-4A71-8BBD-9D65EF03C87C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="87">
   <si>
     <t>Request</t>
   </si>
@@ -34,9 +34,6 @@
     <t>LCL 01724034442</t>
   </si>
   <si>
-    <t>LCL 01316178945</t>
-  </si>
-  <si>
     <t>LCL 01779398037</t>
   </si>
   <si>
@@ -203,9 +200,6 @@
   </si>
   <si>
     <t xml:space="preserve">8801724034442, GP 2560MB, SMSMT, 06/06/2026 10:09:30, [48231 29700639], NALCHITY, JHALOKATHI, IMEI: 352931900461140, IMSI: 470010499560912 [GP] | </t>
-  </si>
-  <si>
-    <t>MSISDN: 8801316178945, LastActiveDateTime: 2026-06-07 22:30:50, LACID: 48261, CellID: 35855137, Latitude: 22.658194, Longitude: 90.344889, Address: 13, PARARA ROAD, P.S. KOTOWALI, DIST. BARISAL, CS Status: Idle [GP]</t>
   </si>
   <si>
     <t xml:space="preserve">8801779398037, 4750, SMSMT, 07/06/2026 23:25:34, [56312 25735199], HOLDING NO. 54/1, FAKIRAPUL, DHAKA, IMEI: 359127131839920, IMSI: 470010441603444 [GP] | </t>
@@ -856,10 +850,10 @@
     <xf numFmtId="0" fontId="13" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -928,8 +922,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}" name="Table1" displayName="Table1" ref="B1:D46" totalsRowShown="0">
-  <autoFilter ref="B1:D46" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}" name="Table1" displayName="Table1" ref="B1:D45" totalsRowShown="0">
+  <autoFilter ref="B1:D45" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}"/>
   <tableColumns count="3">
     <tableColumn id="2" xr3:uid="{2D7AC2AD-014A-48FF-95F7-9CC4728A926F}" name="Request" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{3864D13E-23B2-4E39-A10E-6D64B9F5D0CF}" name="Reply" dataDxfId="0"/>
@@ -1256,7 +1250,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="2" max="2" width="19.08984375" style="1" customWidth="1"/>
@@ -1266,7 +1260,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A1" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1275,7 +1269,7 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="59" x14ac:dyDescent="0.75">
@@ -1286,7 +1280,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="29.5" x14ac:dyDescent="0.75">
@@ -1297,7 +1291,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
@@ -1308,7 +1302,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
@@ -1319,29 +1313,29 @@
         <v>5</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="59" x14ac:dyDescent="0.75">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A7" s="5">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
@@ -1349,32 +1343,32 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A9" s="5">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.75">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="59" x14ac:dyDescent="0.75">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="59" x14ac:dyDescent="0.75">
@@ -1382,43 +1376,43 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A12" s="4">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.75">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="59" x14ac:dyDescent="0.75">
       <c r="A13" s="5">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A14" s="4">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
@@ -1426,98 +1420,98 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A16" s="4">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="59" x14ac:dyDescent="0.75">
       <c r="A17" s="5">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A18" s="4">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="59" x14ac:dyDescent="0.75">
       <c r="A19" s="5">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
       <c r="A20" s="4">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A21" s="5">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.75">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A22" s="4">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A23" s="5">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.75">
@@ -1525,43 +1519,43 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="59" x14ac:dyDescent="0.75">
       <c r="A25" s="5">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
       <c r="A26" s="4">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="59" x14ac:dyDescent="0.75">
       <c r="A27" s="5">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="59" x14ac:dyDescent="0.75">
@@ -1569,10 +1563,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="59" x14ac:dyDescent="0.75">
@@ -1580,46 +1574,46 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A30" s="4">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="59" x14ac:dyDescent="0.75">
       <c r="A31" s="5">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="132.75" x14ac:dyDescent="0.75">
       <c r="A32" s="4">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+    <row r="33" spans="1:4" ht="118" x14ac:dyDescent="0.75">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -1630,7 +1624,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+    <row r="34" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -1641,7 +1635,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+    <row r="35" spans="1:4" ht="118" x14ac:dyDescent="0.75">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -1652,7 +1646,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+    <row r="36" spans="1:4" ht="147.5" x14ac:dyDescent="0.75">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -1663,7 +1657,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="147.5" x14ac:dyDescent="0.75">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -1685,7 +1679,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="39" spans="1:4" ht="59" x14ac:dyDescent="0.75">
       <c r="A39" s="5">
         <v>38</v>
       </c>
@@ -1696,65 +1690,65 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+    <row r="40" spans="1:4" ht="118" x14ac:dyDescent="0.75">
       <c r="A40" s="4">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
       <c r="A41" s="5">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A42" s="4">
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.75">
+        <v>82</v>
+      </c>
+      <c r="D42" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="103.25" x14ac:dyDescent="0.75">
       <c r="A43" s="5">
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D43" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="103.25" x14ac:dyDescent="0.75">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
       <c r="A44" s="4">
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="103.25" x14ac:dyDescent="0.75">
       <c r="A45" s="5">
         <v>44</v>
       </c>
@@ -1762,18 +1756,7 @@
         <v>80</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="103.25" x14ac:dyDescent="0.75">
-      <c r="A46" s="4">
-        <v>45</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backup: uncommitted VPS-only work before pulling security-hardening branch
</commit_message>
<xml_diff>
--- a/Training Data/Automation/LCL.xlsx
+++ b/Training Data/Automation/LCL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\SMS_Automation\Training Data\Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78C767D-7DE7-4CE9-8D2B-9937C6CBFBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECBD642C-916B-4A71-8BBD-9D65EF03C87C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LCL" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="139">
-  <si>
-    <t>SL No</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="87">
   <si>
     <t>Request</t>
   </si>
@@ -31,412 +28,309 @@
     <t>Reply</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>LCL 01617610134</t>
   </si>
   <si>
-    <t>MSISDN: 8801617610134, MSISDN B Party: 8801723599495, Last Call location: Ward No 24, BARISAL SADAR KOTWALI, Barisal, LAC ID: 8005, Cell ID: 28196, Lat_Long: 22.66143, 90.3495, Date_time: 20260607205630, IMEI: 860068048764800, IMSI: 470075012337288 [Robi] | RADIO LOCATION: Ward No-24, Barisal Sadar (kotwali), Barisal, LAC ID: 8005, CELL ID: 28196, LAT, LONG: 22.66143, 90.3495, MS STATUS: Attached, LAST ACTION TIME: 2026-06-07 21:37:12 [Robi]</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>LCL 01724034442</t>
   </si>
   <si>
-    <t>8801724034442, GP 2560MB, SMSMT, 06/06/2026 10:09:30, [48231 29700639], NALCHITY, JHALOKATHI, IMEI: 352931900461140, IMSI: 470010499560912 [GP] | No RL Info Found of 1724034442 [GP]</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>LCL 01316178945</t>
-  </si>
-  <si>
-    <t>8801316178945 / 8801323428959, MTC, 07/06/2026 19:49:15, [23093 53640], PASCHIM CHAR DAPDAPIA, DAPDAPIA, NALCHITY, JHALOKATI, IMEI: 868236085902400, IMSI: 470010491153713 [GP] | MSISDN: 8801316178945, LastActiveDateTime: 2026-06-07 22:30:50, LACID: 48261, CellID: 35855137, Latitude: 22.658194, Longitude: 90.344889, Address: 13, PARARA ROAD, P.S. KOTOWALI, DIST. BARISAL, CS Status: Idle [GP]</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>LCL 01779398037</t>
   </si>
   <si>
-    <t>8801779398037, 4750, SMSMT, 07/06/2026 23:25:34, [56312 25735199], HOLDING NO. 54/1, FAKIRAPUL, DHAKA, IMEI: 359127131839920, IMSI: 470010441603444 [GP] | MSISDN: 8801779398037, LastActiveDateTime: 2026-06-07 23:35:36, LACID: 56312, CellID: 25850635, Latitude: 23.735361, Longitude: 90.416222, Address: 38, NAYAPALTAN, DHAKA-1000, CS Status: Idle [GP]</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>LCL 01312123075</t>
   </si>
   <si>
     <t>8801312123075 / 8801620479563, MTC, 07/06/2026 14:01:06, [27007 22290], VILL ANGARIA, P.O ANGARIA BONDOR, UNION 4 ANGARIA, P.S. DUMKI, PATUAKHALI, IMEI: 357146190845460, IMSI: 470010318024314 [GP]</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>LCL 01620479563</t>
   </si>
   <si>
     <t>MSISDN: 8801620479563, MSISDN B Party: 8801621603027, Last Call location: Vill Bhorpasha, PS Bakerganj, Barishal, LAC ID: 8005, Cell ID: 3610, Lat_Long: 22.5189, 90.343, Date_time: 20260608011153, IMEI: 354680100182050, IMSI: 470075028693785 [Robi]</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
     <t>LCL 01775494991</t>
   </si>
   <si>
     <t>8801775494991 / 8801755370218, MTC, 03/06/2026 15:18:11, [46361 28989246], VILL P.O DHAMURA, UNION SHOLOK, P.S UZIRPUR, DIST BARISAL, IMEI: 868126062531170, IMSI: 470010444160092 [GP]</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>LCL 01333061009</t>
   </si>
   <si>
     <t>8801333061009, GP 35MIN, SMSMT, 03/06/2026 11:08:05, [46361 28989200], VILL P.O DHAMURA, UNION SHOLOK, P.S UZIRPUR, DIST BARISAL, IMEI: 868126062531160, IMSI: 470010426256901 [GP]</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
     <t>LCL 01755370218</t>
   </si>
   <si>
     <t>(B-party of 01775494991 - included in batch reply above)</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>LCL 01958395882</t>
   </si>
   <si>
     <t>MSISDN: 8801958395882, Datetime: 20260608104540, LAC ID: 673, Cell ID: 47113, Address: Vill: Omorpur, Post: Bhuiyarhat, PS: Charfashio, Dist: Bhola, BPARTY: 8801901900977, IMEI: 354388221566410, IMSI: 470039215027744, UsageType: SMSMT, NetworkType: 2G. - Banglalink</t>
   </si>
   <si>
-    <t>11</t>
-  </si>
-  <si>
     <t>LCL 01931270994</t>
   </si>
   <si>
     <t>MSISDN: 8801931270994, Datetime: 20260607122312, LAC ID: 6030, Cell ID: 15425873, Address: Barothi Bazar, Gaurnadi, Barisal, BPARTY: 880424c204468616, IMEI: 350789590248680, IMSI: 470039926367303, UsageType: SMSMT, NetworkType: 4G. - Banglalink</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
     <t>LCL 01567847825</t>
   </si>
   <si>
     <t>(No reply visible in loaded messages)</t>
   </si>
   <si>
-    <t>13</t>
-  </si>
-  <si>
     <t>LCL 01811426571</t>
   </si>
   <si>
     <t>MSISDN: 8801811426571, MSISDN B Party: 4A686F74706F744C6F61, Last Call location: Ward No 46 Part, Hazaribagh, Dhaka, LAC ID: 407, Cell ID: 46478, Lat_Long: 23.75, 90.3448, Date_time: 20260608140235, IMEI: 351207980537560, IMSI: 470022557928135 [Robi]</t>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
     <t>LCL 01730911057</t>
   </si>
   <si>
     <t>8801730911057, GP 45MIN, SMSMT, 08/06/2026 13:27:23, [21034 42832], NEAR BASILA GARDEN CITY PLAY GROUND, MOHAMMADPUR, IMEI: 351207980537570, IMSI: 470010314611892 [GP]</t>
   </si>
   <si>
-    <t>15</t>
-  </si>
-  <si>
     <t>LCL 01750193604</t>
   </si>
   <si>
     <t>8801750193604 / 8801337510464, MTC, 04/06/2026 16:33:43, [23022 50587], RAMNAGAR, MAHESHPUR, BAKORGANJ, BARISAL, IMEI: 865455059456460, IMSI: 470010513871161 [GP]</t>
   </si>
   <si>
-    <t>16</t>
-  </si>
-  <si>
     <t>LCL 01862303409</t>
   </si>
   <si>
     <t>(Part of Mahendigang batch - reply not separately visible)</t>
   </si>
   <si>
-    <t>17</t>
-  </si>
-  <si>
     <t>LCL 01612268083</t>
   </si>
   <si>
     <t>MSISDN: 8801612268083, MSISDN B Party: 8801903311869, Last Call location: Kashipur, Narayanganj Sadar, Narayanganj, LAC ID: 30024, Cell ID: 7842, Lat_Long: 23.60738, 90.491606, Date_time: 20260607012317, IMEI: 351600344667680, IMSI: 470075031845935 [Robi]</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
     <t>LCL 01719698577</t>
   </si>
   <si>
     <t>8801719698577 / 8801732454040, MOC, 08/06/2026 12:26:22, [48251 35844643], ANEX BHABAN, BARISAL CITY CORPORATION, BIBIRPUKUR, BARISAL SADAR, BARISAL, IMEI: 868477051245710, IMSI: 470010494597953 [GP]</t>
   </si>
   <si>
-    <t>19</t>
-  </si>
-  <si>
     <t>LCL 01919904263</t>
   </si>
   <si>
     <t>MN: 01919904263 No Radio Location Found. - Banglalink | MSISDN: 8801919904263, Datetime: 20260605152339, LAC ID: 680, Cell ID: 46521, Address: Vill: Hayatsar, PO: Churamon, PS: Kawnia, Dist: Barisal, IMEI: 864434060146480, IMSI: 470039934828149, NetworkType: 2G. - Banglalink</t>
   </si>
   <si>
-    <t>20</t>
-  </si>
-  <si>
     <t>LCL 01315607014</t>
   </si>
   <si>
     <t>8801315607014 / 8801717167974, MTC, 09/06/2026 00:13:20, [21037 46256], 182/1, EAST TEJTURI BAZAR, TEJGAON, DHAKA, IMSI: 470010459858472 [GP]</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
     <t>LCL 01760675453</t>
   </si>
   <si>
     <t>Sorry No records found against this number 1760675453 [GP]</t>
   </si>
   <si>
-    <t>22</t>
-  </si>
-  <si>
     <t>LCL 01758696171</t>
   </si>
   <si>
     <t>8801758696171, 4750, SMSMT, 22/04/2026 17:47:00, [46501 28984589], KOLCHORI SHAMRAI, CHANPUR, MAHENDIGANJ, BARISAL, IMEI: 353522649744610, IMSI: 470010632925146 [GP]</t>
   </si>
   <si>
-    <t>23</t>
-  </si>
-  <si>
     <t>LCL 01310648009</t>
   </si>
   <si>
     <t>Sorry No records found against this number 1310648009 [GP]</t>
   </si>
   <si>
-    <t>24</t>
-  </si>
-  <si>
     <t>LCL 01721305809</t>
   </si>
   <si>
     <t>Sorry No records found against this number 1721305809 [GP]</t>
   </si>
   <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>LCL 01741989106</t>
-  </si>
-  <si>
-    <t>(LCL 01711989106 - reply not visible)</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>LCL 01863308890</t>
-  </si>
-  <si>
-    <t>(Reply not visible for this request)</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>LCL 01345636569</t>
-  </si>
-  <si>
-    <t>8801345636569 / 8801610656389, MTC, 09/06/2026 13:29:03, [25049 11311], ADAMJEE ROAD (IQBAL GROUP OF INDUSTRIES), P.S: SHIDDHIRGANJ, NARAYANGANJ, IMEI: 861407080007970, IMSI: 470010507001900 [GP]</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>LCL 01715116016</t>
-  </si>
-  <si>
-    <t>8801715116016 / 8801798460306, MTC, 09/06/2026 23:50:36, [23047 13696], 108/102 NATUN BAZAR, BARISHAL, BARISHAL SADAR, BARISAL, IMEI: 860366069821140, IMSI: 470010553967042 [GP] | MSISDN: 8801715116016, LastActiveDateTime: 2026-06-10 00:23:42, LACID: 46331, CellID: 35873311, Latitude: 22.805417, Longitude: 90.309056, Address: FACULTY OF ANIMAL SCIENCE AND VETERINARY MEDICINE BUILDING, RAHOMOTPUR, BABUGANJ, BARISAL, CS Status: Idle [GP]</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
     <t>LCL 01911152692</t>
   </si>
   <si>
     <t>MSISDN: 8801911152692, Datetime: 20260609104730, LAC ID: 680, Cell ID: 60282, Address: Vill - Kandihar, Thana - Banaripara, District - Barisal, BPARTY: 880624B617368, IMEI: 354496311003140, IMSI: 470037400048620, UsageType: SMSMT, NetworkType: 2G. - Banglalink</t>
   </si>
   <si>
-    <t>30</t>
-  </si>
-  <si>
     <t>LCL 01711207942</t>
   </si>
   <si>
     <t>8801711207942, MyGP, SMSMT, 09/06/2026 10:47:36, [46341 29604875], BANORIPARA, BARISAL, IMEI: 354496311038860, IMSI: 470010440738577 [GP]</t>
   </si>
   <si>
-    <t>31</t>
-  </si>
-  <si>
     <t>LCL 01631371920</t>
   </si>
   <si>
     <t>MSISDN: 8801631371920, MSISDN B Party: Airtel, Last Call location: vill Tetla, P O Tetla, Banaripara, Barishal, LAC ID: 820043, Cell ID: 75, Lat_Long: 22.81357, 90.08629, Date_time: 20260605072416, IMEI: 862410074377150, IMSI: 470075005033851 [Robi]</t>
   </si>
   <si>
-    <t>32</t>
-  </si>
-  <si>
     <t>LCL 01711351928</t>
   </si>
   <si>
     <t>8801711351928, Navana Land, SMSMT, 10/06/2026 10:15:20, [62411 40979232], MUNICIPAL HOLDING NO. 59/B/1, ROY J. C. GUHA ROAD, KRISHTOPUR, P.S MYMENSINGH SADAR, MYMENSINGH, IMEI: 862365044189750, IMSI: 470010513636040 [GP]</t>
   </si>
   <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>LCL 01888002490</t>
-  </si>
-  <si>
-    <t>(Split from multi-number request LCL 01888002490 01333821028 - reply not separately shown)</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>LCL 01333821028</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
     <t>LCL 01937344944</t>
   </si>
   <si>
     <t>MSISDN: 8801937344944, Datetime: 20260608111805, LAC ID: 461, Cell ID: 41753, Address: House No: 105/22k, Thana Road, PS: Sonadanga, Dist: Khulna, BPARTY: 8801938773957, IMEI: 359498701015280, IMSI: 470039946221263, UsageType: MTC, NetworkType: 2G. - Banglalink</t>
   </si>
   <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>LCL 01623766981</t>
-  </si>
-  <si>
-    <t>(No reply visible for this request)</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>LCL 01720542190</t>
-  </si>
-  <si>
-    <t>8801720542190 / 8801725927837, MOC, 10/06/2026 09:48:00, [23126 50574], VILL KADIRABAD, P.O KADIRABAD, UNION LATA, P.S MAHENDIGANJ, BARISAL, IMEI: 344685625789860, IMSI: 470010383180005 [GP]</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
     <t>LCL 01703520704</t>
   </si>
   <si>
     <t>8801703520704, GP, SMSMT, 09/06/2026 18:13:41, [46301 28995871], VILL-GABIKHOLA, P.O-GARURIA, P/S-BAKERGONJ, BARISAL, IMEI: 866446059282170, IMSI: 470010491639968 [GP]</t>
   </si>
   <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>LCL 01602-389949</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>LCL 01719182914</t>
-  </si>
-  <si>
-    <t>8801719182914 / 8801789360756, MTC, 09/06/2026 23:10:54, [23126 29095], PATTANI BHANGAR CHAR, GUABARIA, HIZLA, BARISHAL, IMSI: 470010352788437 [GP]</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>43</t>
-  </si>
-  <si>
-    <t>LCL 01757265392</t>
-  </si>
-  <si>
-    <t>(Split from 5-number batch: LCL 01757265392 01844468499 01768233922 01736373112 01757232333 - system returned batch reply for these numbers)</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>LCL 01844468499</t>
-  </si>
-  <si>
-    <t>(Split from 5-number batch - see above)</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>LCL 01768233922</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>LCL 01736373112</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>LCL 01757232333</t>
-  </si>
-  <si>
-    <t>8801724761972 / 8801325397520, MTC, 10/06/2026 21:58:49, [22049 50739], MOUZA-BANARIPARA, SADAR ROAD, 3 NO WORD, BANARIPARA, BARISHAL, IMEI: 350419993156990, IMSI: 470010081907258 [GP]</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
     <t>LCL 01319472535</t>
   </si>
   <si>
-    <t>MSISDN: 8801319472535, LastActiveDateTime: 2026-06-10 12:31:29, LACID: 23066, CellID: 22578, Latitude: 23.371472, Longitude: 90.034444, Address: VILL.- RASHIBPURA, MALIGRAM BAZAR, MOUZA-MALIGRAM, VANGA, FARIDPUR, CS Status: Idle, Volte Status: N/A [GP] | 8801319472535, GP, SMSMT, 10/06/2026 12:31:17, [48271 28698401], VILL: PULIA, P.O: CHANDRA BAZAR, UNION: CHANDRA, P.S: BHANGA, FARIDPUR, IMEI: 357726270741110, IMSI: 470010402936218 [GP]</t>
+    <t>MSISDN: 8801617610134, MSISDN B Party: 8801723599495, Last Call location: Ward No 24, BARISAL SADAR KOTWALI, Barisal, LAC ID: 8005, Cell ID: 28196, Lat_Long: 22.66143, 90.3495, Date_time: 20260607205630, IMEI: 860068048764800, IMSI: 470075012337288 [Robi] |</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8801724034442, GP 2560MB, SMSMT, 06/06/2026 10:09:30, [48231 29700639], NALCHITY, JHALOKATHI, IMEI: 352931900461140, IMSI: 470010499560912 [GP] | </t>
+  </si>
+  <si>
+    <t xml:space="preserve">8801779398037, 4750, SMSMT, 07/06/2026 23:25:34, [56312 25735199], HOLDING NO. 54/1, FAKIRAPUL, DHAKA, IMEI: 359127131839920, IMSI: 470010441603444 [GP] | </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSISDN: 8801319472535, LastActiveDateTime: 2026-06-10 12:31:29, LACID: 23066, CellID: 22578, Latitude: 23.371472, Longitude: 90.034444, Address: VILL.- RASHIBPURA, MALIGRAM BAZAR, MOUZA-MALIGRAM, VANGA, FARIDPUR, CS Status: Idle, Volte Status: N/A [GP] | </t>
+  </si>
+  <si>
+    <t>LCL 01864591168</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801864591168
+MSISDN B Party: 8801821764035
+Last Call location: Castle Green,H  142,Green Road,,Farmgate,Dhaka 1215
+LAC ID: 108
+Cell ID: 897
+Lat_Long: 23.7535, 90.3882
+Date_time: 20260615204215
+IMEI: 869727086437610
+IMSI: 470022563349762 [Robi]</t>
+  </si>
+  <si>
+    <t>LCL 01305424184</t>
+  </si>
+  <si>
+    <t>8801305424184
+8801933640177
+MOC
+15/06/2026 09:26:42
+[23117 22339]
+MOUZA NAGARBAKA,  P.S. &amp;amp; SUB REGISTRY OFFICE MIRPUR,  DIST. KUSTIA.
+866941062115380
+470010485077007 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01721586862</t>
+  </si>
+  <si>
+    <t>8801721586862
+8801932161211
+MTC
+15/06/2026 20:32:11
+[23011 21691]
+BISWAS BARI, VILL-LOKKHIKOL,  P.S. JHENAIDAH SADAR,  JHENAIDAH JHENAIDAH SADAR  JHENAIDAH
+358564994871350
+470010483500257 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01744708168</t>
+  </si>
+  <si>
+    <t>8801744708168
+bKash
+SMSMT
+14/06/2026 19:57:22
+[21025 12297]
+VILL: SHEMPUR  HEMAYETPUR PS: SAVER  DIST: DHAKA
+353973860706950
+470010369479393 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01836526001</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801836526001
+MSISDN B Party: 5370656369616C506163
+Last Call location: Vill  Purbakandi Paschimpar, P O  Uttar Char   8270, P S  Mehendiganj, Dist  Barisal
+LAC ID: 8006
+Cell ID: 28390
+Lat_Long: 22.85657, 90.54667
+Date_time: 20251202132329
+IMEI: 866254085016420
+IMSI: 470022595759345 [Robi]</t>
+  </si>
+  <si>
+    <t>LCL 01994076892</t>
+  </si>
+  <si>
+    <t>MSISDN: 01994076892 No Data Available within 90 Days (LCL) - Banglalink</t>
+  </si>
+  <si>
+    <t>LCL 01759778356</t>
+  </si>
+  <si>
+    <t>Sorry No records found against this number 1759778356 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01938218511</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801938218511, Datetime: 20260615224027, LAC ID: 1202, Cell ID: 3012355, Address: Md. Abul Kashem, 311 south Monipur (Mollapara), Near Kuwaity mosque, Mirpur-2, BPARTY: 880811660038123, IMEI: 350347640688710, IMSI: 470039954420135, UsageType: MTC, NetworkType: 4G. - Banglalink</t>
+  </si>
+  <si>
+    <t>LCL 01309821052</t>
+  </si>
+  <si>
+    <t>8801309821052
+8801729558492
+MOC
+15/06/2026 17:13:57
+[23047 50689]
+APON NIBASH, HOUSE NO# 502, ROAD- AGARPUR,BARISHAL SADAR,BARISHAL SADAR,BARISHAL
+356008090251500
+470010482120610 [GP]</t>
+  </si>
+  <si>
+    <t>LCL 01340484381</t>
+  </si>
+  <si>
+    <t>LCL 01869033806</t>
+  </si>
+  <si>
+    <t>Sorry No records found against this number 1869033806 [GP]</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>**Look this number is robi but msg sent to gp. So no record replied</t>
+  </si>
+  <si>
+    <t>8801340484381
+8801847348716
+SMSMT
+16/06/2026 13:31:07
+[48251 2244188]
+866183068507830
+470010977470798 [GP]</t>
+  </si>
+  <si>
+    <t>SL NO</t>
   </si>
 </sst>
 </file>
@@ -579,7 +473,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -759,8 +653,20 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -875,6 +781,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -920,16 +839,22 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -976,15 +901,12 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1000,12 +922,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}" name="Table1" displayName="Table1" ref="A1:C49" totalsRowShown="0">
-  <autoFilter ref="A1:C49" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}" name="Table1" displayName="Table1" ref="B1:D45" totalsRowShown="0">
+  <autoFilter ref="B1:D45" xr:uid="{CC6C1350-271C-41C0-80E9-E79C32EC99D0}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{325C3C9D-4760-4419-9DD2-AB65634C7B08}" name="SL No" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{2D7AC2AD-014A-48FF-95F7-9CC4728A926F}" name="Request" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{3864D13E-23B2-4E39-A10E-6D64B9F5D0CF}" name="Reply" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{3C8B4891-26D5-4D39-A506-E466FD96FCE7}" name="Column1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1328,551 +1250,513 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="A1:D45"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="8.83984375" style="1"/>
-    <col min="2" max="2" width="19.1015625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="62.7890625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="19.08984375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="69.54296875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="51.58984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A1" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="100.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="1" t="s">
+      <c r="C2" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C3" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C4" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+    </row>
+    <row r="6" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="86.4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="1" t="s">
+    <row r="7" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="86.4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="1" t="s">
+    <row r="10" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="3" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="2" t="s">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="1" t="s">
+    <row r="13" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A13" s="5">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="3" t="s">
+    </row>
+    <row r="14" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="1" t="s">
+      <c r="C14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="2" t="s">
+    </row>
+    <row r="15" spans="1:4" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A15" s="5">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="1" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="3" t="s">
+    </row>
+    <row r="17" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A17" s="5">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="1" t="s">
+      <c r="C17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="2" t="s">
+    </row>
+    <row r="18" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="1" t="s">
+    <row r="19" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A19" s="5">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="3" t="s">
+    </row>
+    <row r="20" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="1" t="s">
+      <c r="C20" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="2" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A21" s="5">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C21" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="1" t="s">
+    <row r="22" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A22" s="4">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="3" t="s">
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A23" s="5">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="1" t="s">
+      <c r="C23" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="2" t="s">
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A24" s="4">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C24" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="1" t="s">
+    <row r="25" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A25" s="5">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="3" t="s">
+    </row>
+    <row r="26" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="2" t="s">
+    </row>
+    <row r="27" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A27" s="5">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C27" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="1" t="s">
+    <row r="28" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="3" t="s">
+    </row>
+    <row r="29" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A29" s="5">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="1" t="s">
+      <c r="C29" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="2" t="s">
+    </row>
+    <row r="30" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A30" s="4">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C30" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="1" t="s">
+    <row r="31" spans="1:3" ht="59" x14ac:dyDescent="0.75">
+      <c r="A31" s="5">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B21" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="3" t="s">
+    </row>
+    <row r="32" spans="1:3" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A32" s="4">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="1" t="s">
+      <c r="C32" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="2" t="s">
+    </row>
+    <row r="33" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+      <c r="A33" s="5">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C33" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="1" t="s">
+    <row r="34" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A34" s="4">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="3" t="s">
+    </row>
+    <row r="35" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+      <c r="A35" s="5">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="1" t="s">
+      <c r="C35" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B24" s="2" t="s">
+    </row>
+    <row r="36" spans="1:4" ht="147.5" x14ac:dyDescent="0.75">
+      <c r="A36" s="4">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C36" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="1" t="s">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A37" s="5">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="3" t="s">
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A38" s="4">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="1" t="s">
+      <c r="C38" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B26" s="2" t="s">
+    </row>
+    <row r="39" spans="1:4" ht="59" x14ac:dyDescent="0.75">
+      <c r="A39" s="5">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C39" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="1" t="s">
+    <row r="40" spans="1:4" ht="118" x14ac:dyDescent="0.75">
+      <c r="A40" s="4">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A41" s="5">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C27" s="3" t="s">
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="A42" s="4">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D42" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="103.25" x14ac:dyDescent="0.75">
+      <c r="A43" s="5">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="100.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B29" s="2" t="s">
+      <c r="C43" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B34" s="2" t="s">
+    </row>
+    <row r="44" spans="1:4" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A44" s="4">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C34" s="3" t="s">
+    </row>
+    <row r="45" spans="1:4" ht="103.25" x14ac:dyDescent="0.75">
+      <c r="A45" s="5">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" ht="100.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>138</v>
+      <c r="C45" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>